<commit_message>
Add Registry_Gaps sheet to objects audit workbook
Captures 21 gaps found by AST-precise scan of cursor.execute() calls and
mockdata SQL: 9 setup tables used in code but not in object registry
(homepage_assignment, page_builder, page_component, whatsapp_message,
user_group_profiles, user_group_public_groups, otp_verification_sessions,
tenant_provisioning_errors, organizations), 3 missing business objects,
2 naming inconsistencies (dashboard_folder vs _folders, reports/report/
report_folder), 2 typos (organization in pdfgen, hsitory), 4 legacy
duplicates (customers/products/invoices/invoice_items), and 1 Django
model with no registry row (facebookleadwebhooks).

https://claude.ai/code/session_01PQe7UPAGCLLjpH2CtVo1VY
</commit_message>
<xml_diff>
--- a/objects_audit.xlsx
+++ b/objects_audit.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="All_Objects" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Migration_Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Registry_Gaps" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +58,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B084"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -101,6 +117,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -218,6 +243,20 @@
     <tableColumn id="7" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RegistryGaps" displayName="RegistryGaps" ref="A1:E22" headerRowCount="1">
+  <autoFilter ref="A1:E22"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Kind"/>
+    <tableColumn id="2" name="Table / Item"/>
+    <tableColumn id="3" name="Label / Note"/>
+    <tableColumn id="4" name="Evidence (file:line)"/>
+    <tableColumn id="5" name="Recommended Action"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showRowStripes="0"/>
 </table>
 </file>
 
@@ -510,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -658,6 +697,101 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Primary migration scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REGISTRY GAPS (from AST scan + .sql review)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Missing business object</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Naming inconsistency</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bug — likely typo</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Legacy duplicate</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Django-modeled, not in registry</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Total registry gaps</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>21</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>See Registry_Gaps sheet</t>
         </is>
       </c>
     </row>
@@ -14299,4 +14433,622 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="73" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Table / Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Label / Note</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence (file:line)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>homepage_assignment</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Homepage Assignment</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>api/ORM/setup/newprofile.py:88,93</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); will be migrated to Django ORM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>organizations</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Organizations</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>adminuser/services/organizations.py:28,53; api/models.py:Organization</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); already has Django model</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>otp_verification_sessions</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>OTP Verification Sessions</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>public/auth/otp_verification.py:156,198</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); auth/OTP flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>page_builder</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Page Builder</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>api/ORM/setup/update_page_builder.py:28</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); distinct from registered 'page_builder_assignment'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>page_component</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Page Component</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>api/ORM/setup/update_page_builder.py:66,78</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); page-builder child table</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>tenant_provisioning_errors</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Tenant Provisioning Errors</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>public/utils/error_log.py:20</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); tenant onboarding error log</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>user_group_profiles</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>User Group Profiles</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>utils/usergroup_utils.py:305</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); junction table for user_group &lt;-&gt; profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>user_group_public_groups</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>User Group Public Groups</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>utils/usergroup_utils.py:317; api/workflows/workflow_executor.py:552</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); junction for nested user groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Missing setup table</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>whatsapp_message</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>WhatsApp Message</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>api/BL/whatsapp/utils.py:18,67</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=TRUE); chat-message store</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Missing business object</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>dashboard_component</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard Component</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>sqlfiles/mockdata/reports.sql</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Add registry row; child of dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Missing business object</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>dashboard_folders</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard Folders</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>sqlfiles/mockdata/reports.sql</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Plural form referenced; registry has 'dashboard_folder' singular - pick one and reconcile</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Missing business object</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>report_folder</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Report Folder</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>sqlfiles/mockdata/reports.sql</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Add registry row (setup=FALSE); related to 'reports' (already registered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Naming inconsistency</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>dashboard_folder vs dashboard_folders</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard Folder</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>registry: dashboard_folder (singular); code: dashboard_folders (plural)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Standardize on one form across registry, code, and mockdata</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Naming inconsistency</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>reports vs report vs report_folder</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>registry: 'reports'; code uses 'report' and 'report_folder' too</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Standardize and register all related tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Bug — likely typo</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>hsitory</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Probably means 'history'</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>registry row in objects.sql</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Rename to 'history' before migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Bug — likely typo</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>organization (singular)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Probably means 'organizations'</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>api/pdfgen/views.py:74</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Fix the SQL string to use 'organizations'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Legacy duplicate</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>customers (setup) vs customer (business)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>objects.sql registers both</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Investigate which is actually used; merge or delete the unused one</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Legacy duplicate</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>invoice_items (setup) vs invoice_item (business)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Item</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>objects.sql registers both</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Investigate which is actually used; merge or delete the unused one</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Legacy duplicate</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>invoices (setup) vs invoice (business)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>objects.sql registers both</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Investigate which is actually used; merge or delete the unused one</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Legacy duplicate</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>products (setup) vs product (business)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>objects.sql registers both</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Investigate which is actually used; merge or delete the unused one</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Django-modeled, not in registry</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>facebookleadwebhooks</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Facebook Lead Webhooks</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>facebook/models.py (currently commented out)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Add registry row OR delete the Django model — currently dead code</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>